<commit_message>
dbn-08-20-25 - mapping done
</commit_message>
<xml_diff>
--- a/ASCal/template.xlsx
+++ b/ASCal/template.xlsx
@@ -3369,7 +3369,7 @@
     <cellStyle name="Normal 4" xfId="4"/>
     <cellStyle name="Normal 5" xfId="5"/>
   </cellStyles>
-  <dxfs count="142">
+  <dxfs count="144">
     <dxf>
       <fill>
         <patternFill>
@@ -3472,6 +3472,26 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8053,28 +8073,28 @@
       <c r="H70" s="238"/>
       <c r="I70" s="238" t="str">
         <f>CONCATENATE(DataSheet!L55," ",DataSheet!P55)</f>
-        <v xml:space="preserve"> mV</v>
+        <v>60 mV</v>
       </c>
       <c r="J70" s="238"/>
       <c r="K70" s="238"/>
       <c r="L70" s="238"/>
-      <c r="M70" s="238" t="e">
+      <c r="M70" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AM55,"0.0")," ",DataSheet!P55)</f>
-        <v>#DIV/0!</v>
+        <v>60.0 mV</v>
       </c>
       <c r="N70" s="238"/>
       <c r="O70" s="238"/>
       <c r="P70" s="238"/>
-      <c r="Q70" s="238" t="e">
+      <c r="Q70" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AR55,"0.0")," ",DataSheet!P55)</f>
-        <v>#DIV/0!</v>
+        <v>0.0 mV</v>
       </c>
       <c r="R70" s="238"/>
       <c r="S70" s="238"/>
       <c r="T70" s="238"/>
-      <c r="U70" s="238" t="e">
+      <c r="U70" s="238" t="str">
         <f>CONCATENATE(," ",TEXT(DataSheet!DD55,"0.000")," ",DataSheet!CZ55)</f>
-        <v>#DIV/0!</v>
+        <v xml:space="preserve"> 0.058 mV</v>
       </c>
       <c r="V70" s="238"/>
       <c r="W70" s="238"/>
@@ -8095,21 +8115,21 @@
       <c r="L71" s="238"/>
       <c r="M71" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AM56,"0.0")," ",DataSheet!P56)</f>
-        <v>40.0 mV</v>
+        <v>540.0 mV</v>
       </c>
       <c r="N71" s="238"/>
       <c r="O71" s="238"/>
       <c r="P71" s="238"/>
       <c r="Q71" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AR56,"0.0")," ",DataSheet!P56)</f>
-        <v>-500.0 mV</v>
+        <v>0.0 mV</v>
       </c>
       <c r="R71" s="238"/>
       <c r="S71" s="238"/>
       <c r="T71" s="238"/>
       <c r="U71" s="238" t="str">
         <f>CONCATENATE(," ",TEXT(DataSheet!DD56,"0.000")," ",DataSheet!CZ56)</f>
-        <v xml:space="preserve"> 80.000 mV</v>
+        <v xml:space="preserve"> 0.058 mV</v>
       </c>
       <c r="V71" s="238"/>
       <c r="W71" s="238"/>
@@ -8916,14 +8936,14 @@
       <c r="L96" s="257"/>
       <c r="M96" s="257" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AM107,"0.000")," ",DataSheet!P107)</f>
-        <v>5.400 MΩ</v>
+        <v>540.000 MΩ</v>
       </c>
       <c r="N96" s="257"/>
       <c r="O96" s="257"/>
       <c r="P96" s="257"/>
       <c r="Q96" s="257" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AR107,"0.000")," ",DataSheet!P107)</f>
-        <v>0.000 MΩ</v>
+        <v>534.600 MΩ</v>
       </c>
       <c r="R96" s="257"/>
       <c r="S96" s="257"/>
@@ -9307,14 +9327,14 @@
       <c r="L122" s="238"/>
       <c r="M122" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AM76,"0.0")," ",DataSheet!P76)</f>
-        <v>59.4 mV</v>
+        <v>60.3 mV</v>
       </c>
       <c r="N122" s="238"/>
       <c r="O122" s="238"/>
       <c r="P122" s="238"/>
       <c r="Q122" s="238" t="str">
         <f>CONCATENATE(TEXT(DataSheet!AR76,"0.0")," ",DataSheet!P76)</f>
-        <v>-0.6 mV</v>
+        <v>0.3 mV</v>
       </c>
       <c r="R122" s="238"/>
       <c r="S122" s="238"/>
@@ -15907,7 +15927,9 @@
       <c r="I55" s="320"/>
       <c r="J55" s="320"/>
       <c r="K55" s="321"/>
-      <c r="L55" s="297"/>
+      <c r="L55" s="297">
+        <v>60</v>
+      </c>
       <c r="M55" s="298"/>
       <c r="N55" s="298"/>
       <c r="O55" s="298"/>
@@ -15921,32 +15943,38 @@
       <c r="U55" s="301"/>
       <c r="V55" s="301"/>
       <c r="W55" s="301"/>
-      <c r="X55" s="291"/>
+      <c r="X55" s="291">
+        <v>60</v>
+      </c>
       <c r="Y55" s="291"/>
       <c r="Z55" s="291"/>
       <c r="AA55" s="291"/>
       <c r="AB55" s="291"/>
-      <c r="AC55" s="291"/>
+      <c r="AC55" s="291">
+        <v>60</v>
+      </c>
       <c r="AD55" s="291"/>
       <c r="AE55" s="291"/>
       <c r="AF55" s="291"/>
       <c r="AG55" s="291"/>
-      <c r="AH55" s="291"/>
+      <c r="AH55" s="291">
+        <v>60</v>
+      </c>
       <c r="AI55" s="291"/>
       <c r="AJ55" s="291"/>
       <c r="AK55" s="291"/>
       <c r="AL55" s="291"/>
-      <c r="AM55" s="291" t="e">
+      <c r="AM55" s="291">
         <f t="shared" ref="AM55:AM68" si="0">AVERAGE(X55:AL55)</f>
-        <v>#DIV/0!</v>
+        <v>60</v>
       </c>
       <c r="AN55" s="291"/>
       <c r="AO55" s="291"/>
       <c r="AP55" s="291"/>
       <c r="AQ55" s="291"/>
-      <c r="AR55" s="291" t="e">
+      <c r="AR55" s="291">
         <f>AM55-L55</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="AS55" s="291"/>
       <c r="AT55" s="291"/>
@@ -15957,22 +15985,34 @@
       <c r="AY55" s="139"/>
       <c r="AZ55" s="172"/>
       <c r="BA55" s="173"/>
-      <c r="BB55" s="306"/>
+      <c r="BB55" s="306">
+        <f>ABS(AM55*0.1%)+(1*CK55)</f>
+        <v>0.16</v>
+      </c>
       <c r="BC55" s="306"/>
       <c r="BD55" s="306"/>
       <c r="BE55" s="306"/>
       <c r="BF55" s="306"/>
-      <c r="BG55" s="306"/>
+      <c r="BG55" s="306">
+        <f>L55+BB55</f>
+        <v>60.16</v>
+      </c>
       <c r="BH55" s="306"/>
       <c r="BI55" s="306"/>
       <c r="BJ55" s="306"/>
       <c r="BK55" s="306"/>
-      <c r="BL55" s="306"/>
+      <c r="BL55" s="306">
+        <f>L55-BB55</f>
+        <v>59.84</v>
+      </c>
       <c r="BM55" s="306"/>
       <c r="BN55" s="306"/>
       <c r="BO55" s="306"/>
       <c r="BP55" s="306"/>
-      <c r="BQ55" s="292"/>
+      <c r="BQ55" s="292" t="str">
+        <f>IF(AND(AM55&lt;=BG55,AM55&gt;=BL55),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
       <c r="BR55" s="292"/>
       <c r="BS55" s="292"/>
       <c r="BT55" s="292"/>
@@ -16037,9 +16077,9 @@
       <c r="CP55" s="70" t="s">
         <v>70</v>
       </c>
-      <c r="CQ55" s="83" t="e">
+      <c r="CQ55" s="83">
         <f>STDEV(X55:AL55)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="CR55" s="71" t="str">
         <f t="shared" ref="CR55:CR68" si="2">P55</f>
@@ -16049,26 +16089,26 @@
         <f>SQRT(3)</f>
         <v>1.7320508075688772</v>
       </c>
-      <c r="CT55" s="85" t="e">
+      <c r="CT55" s="85">
         <f>CQ55/CS55</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="CU55" s="8"/>
-      <c r="CV55" s="92" t="e">
+      <c r="CV55" s="92">
         <f>SQRT(SUMSQ(CT55,CN55,CH55,CB55))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="CW55" s="88" t="e">
+        <v>2.8870080677638112E-2</v>
+      </c>
+      <c r="CW55" s="88">
         <f>(CV55^4)/(((CT55^4)/2)+((CN55^4)/200)+((CH55^4)/200)+((CB55^4)/200))</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="CX55" s="93" t="e">
+        <v>200.07114799774902</v>
+      </c>
+      <c r="CX55" s="93">
         <f>ROUND(TINV(0.05,CW55),0)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="CY55" s="103" t="e">
+        <v>2</v>
+      </c>
+      <c r="CY55" s="103">
         <f>(CV55*CX55)</f>
-        <v>#DIV/0!</v>
+        <v>5.7740161355276223E-2</v>
       </c>
       <c r="CZ55" s="104" t="str">
         <f t="shared" ref="CZ55:CZ68" si="3">P55</f>
@@ -16082,9 +16122,9 @@
         <f>CZ55</f>
         <v>mV</v>
       </c>
-      <c r="DD55" s="220" t="e">
+      <c r="DD55" s="220">
         <f>MAX(DB55,CY55)</f>
-        <v>#DIV/0!</v>
+        <v>5.7740161355276223E-2</v>
       </c>
       <c r="DE55" s="178" t="s">
         <v>161</v>
@@ -16122,21 +16162,21 @@
       <c r="V56" s="301"/>
       <c r="W56" s="301"/>
       <c r="X56" s="307">
-        <v>60</v>
+        <v>540</v>
       </c>
       <c r="Y56" s="308"/>
       <c r="Z56" s="308"/>
       <c r="AA56" s="308"/>
       <c r="AB56" s="308"/>
       <c r="AC56" s="307">
-        <v>60</v>
+        <v>540</v>
       </c>
       <c r="AD56" s="308"/>
       <c r="AE56" s="308"/>
       <c r="AF56" s="308"/>
       <c r="AG56" s="308"/>
       <c r="AH56" s="307">
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="AI56" s="308"/>
       <c r="AJ56" s="308"/>
@@ -16144,7 +16184,7 @@
       <c r="AL56" s="308"/>
       <c r="AM56" s="307">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>540</v>
       </c>
       <c r="AN56" s="308"/>
       <c r="AO56" s="308"/>
@@ -16152,7 +16192,7 @@
       <c r="AQ56" s="309"/>
       <c r="AR56" s="307">
         <f t="shared" ref="AR56:AR68" si="4">AM56-L56</f>
-        <v>-500</v>
+        <v>0</v>
       </c>
       <c r="AS56" s="308"/>
       <c r="AT56" s="308"/>
@@ -16165,7 +16205,7 @@
       <c r="BA56" s="173"/>
       <c r="BB56" s="306">
         <f t="shared" ref="BB56:BB57" si="5">ABS(AM56*0.1%)+(1*CK56)</f>
-        <v>0.14000000000000001</v>
+        <v>0.64</v>
       </c>
       <c r="BC56" s="306"/>
       <c r="BD56" s="306"/>
@@ -16173,7 +16213,7 @@
       <c r="BF56" s="306"/>
       <c r="BG56" s="291">
         <f t="shared" ref="BG56:BG68" si="6">L56+BB56</f>
-        <v>540.14</v>
+        <v>540.64</v>
       </c>
       <c r="BH56" s="291"/>
       <c r="BI56" s="291"/>
@@ -16181,7 +16221,7 @@
       <c r="BK56" s="291"/>
       <c r="BL56" s="291">
         <f t="shared" ref="BL56:BL68" si="7">L56-BB56</f>
-        <v>539.86</v>
+        <v>539.36</v>
       </c>
       <c r="BM56" s="291"/>
       <c r="BN56" s="291"/>
@@ -16189,7 +16229,7 @@
       <c r="BP56" s="291"/>
       <c r="BQ56" s="292" t="str">
         <f t="shared" ref="BQ56:BQ68" si="8">IF(AND(AM56&lt;=BG56,AM56&gt;=BL56),"PASS","FAIL")</f>
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="BR56" s="292"/>
       <c r="BS56" s="292"/>
@@ -16257,7 +16297,7 @@
       </c>
       <c r="CQ56" s="6">
         <f t="shared" ref="CQ56:CQ68" si="16">STDEV(X56:AL56)</f>
-        <v>34.641016151377549</v>
+        <v>0</v>
       </c>
       <c r="CR56" s="1" t="str">
         <f t="shared" si="2"/>
@@ -16269,24 +16309,24 @@
       </c>
       <c r="CT56" s="86">
         <f t="shared" ref="CT56:CT68" si="18">CQ56/CS56</f>
-        <v>20.000000000000004</v>
+        <v>0</v>
       </c>
       <c r="CU56" s="8"/>
       <c r="CV56" s="94">
         <f t="shared" ref="CV56:CV68" si="19">SQRT(SUMSQ(CT56,CN56,CH56,CB56))</f>
-        <v>20.000020860884955</v>
+        <v>2.8886603007853544E-2</v>
       </c>
       <c r="CW56" s="5">
         <f t="shared" ref="CW56:CW68" si="20">(CV56^4)/(((CT56^4)/2)+((CN56^4)/200)+((CH56^4)/200)+((CB56^4)/200))</f>
-        <v>2.0000083443669494</v>
+        <v>200.52919907372751</v>
       </c>
       <c r="CX56" s="95">
         <f t="shared" ref="CX56:CX57" si="21">ROUND(TINV(0.05,CW56),0)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="CY56" s="105">
         <f t="shared" ref="CY56:CY58" si="22">(CV56*CX56)</f>
-        <v>80.000083443539822</v>
+        <v>5.7773206015707089E-2</v>
       </c>
       <c r="CZ56" s="106" t="str">
         <f t="shared" si="3"/>
@@ -16302,7 +16342,7 @@
       </c>
       <c r="DD56" s="220">
         <f t="shared" ref="DD56:DD71" si="24">MAX(DB56,CY56)</f>
-        <v>80.000083443539822</v>
+        <v>5.7773206015707089E-2</v>
       </c>
       <c r="DE56" s="178" t="str">
         <f t="shared" ref="DE56:DE68" si="25">DC56</f>
@@ -20084,14 +20124,14 @@
       <c r="AA76" s="308"/>
       <c r="AB76" s="309"/>
       <c r="AC76" s="307">
-        <v>59.1</v>
+        <v>60</v>
       </c>
       <c r="AD76" s="308"/>
       <c r="AE76" s="308"/>
       <c r="AF76" s="308"/>
       <c r="AG76" s="309"/>
       <c r="AH76" s="307">
-        <v>59.1</v>
+        <v>60.9</v>
       </c>
       <c r="AI76" s="308"/>
       <c r="AJ76" s="308"/>
@@ -20099,7 +20139,7 @@
       <c r="AL76" s="309"/>
       <c r="AM76" s="307">
         <f t="shared" ref="AM76:AM79" si="59">AVERAGE(X76:AL76)</f>
-        <v>59.4</v>
+        <v>60.300000000000004</v>
       </c>
       <c r="AN76" s="308"/>
       <c r="AO76" s="308"/>
@@ -20107,7 +20147,7 @@
       <c r="AQ76" s="309"/>
       <c r="AR76" s="291">
         <f t="shared" ref="AR76:AR79" si="60">AM76-L76</f>
-        <v>-0.60000000000000142</v>
+        <v>0.30000000000000426</v>
       </c>
       <c r="AS76" s="291"/>
       <c r="AT76" s="291"/>
@@ -20120,7 +20160,7 @@
       <c r="BA76" s="173"/>
       <c r="BB76" s="329">
         <f>(AM76*0.7%)+(4*CK76)</f>
-        <v>0.81579999999999997</v>
+        <v>0.82210000000000005</v>
       </c>
       <c r="BC76" s="329"/>
       <c r="BD76" s="329"/>
@@ -20128,7 +20168,7 @@
       <c r="BF76" s="329"/>
       <c r="BG76" s="329">
         <f t="shared" ref="BG76:BG79" si="61">L76+BB76</f>
-        <v>60.815800000000003</v>
+        <v>60.822099999999999</v>
       </c>
       <c r="BH76" s="329"/>
       <c r="BI76" s="329"/>
@@ -20136,7 +20176,7 @@
       <c r="BK76" s="329"/>
       <c r="BL76" s="329">
         <f t="shared" ref="BL76:BL79" si="62">L76-BB76</f>
-        <v>59.184199999999997</v>
+        <v>59.177900000000001</v>
       </c>
       <c r="BM76" s="329"/>
       <c r="BN76" s="329"/>
@@ -26537,21 +26577,21 @@
       <c r="V107" s="301"/>
       <c r="W107" s="301"/>
       <c r="X107" s="329">
-        <v>5.4</v>
+        <v>540</v>
       </c>
       <c r="Y107" s="329"/>
       <c r="Z107" s="329"/>
       <c r="AA107" s="329"/>
       <c r="AB107" s="329"/>
       <c r="AC107" s="329">
-        <v>5.4</v>
+        <v>540</v>
       </c>
       <c r="AD107" s="329"/>
       <c r="AE107" s="329"/>
       <c r="AF107" s="329"/>
       <c r="AG107" s="329"/>
       <c r="AH107" s="329">
-        <v>5.4</v>
+        <v>540</v>
       </c>
       <c r="AI107" s="329"/>
       <c r="AJ107" s="329"/>
@@ -26559,7 +26599,7 @@
       <c r="AL107" s="329"/>
       <c r="AM107" s="329">
         <f t="shared" ref="AM107" si="169">AVERAGE(X107:AL107)</f>
-        <v>5.4000000000000012</v>
+        <v>540</v>
       </c>
       <c r="AN107" s="329"/>
       <c r="AO107" s="329"/>
@@ -26567,7 +26607,7 @@
       <c r="AQ107" s="329"/>
       <c r="AR107" s="329">
         <f t="shared" ref="AR107" si="170">AM107-L107</f>
-        <v>0</v>
+        <v>534.6</v>
       </c>
       <c r="AS107" s="329"/>
       <c r="AT107" s="329"/>
@@ -26580,7 +26620,7 @@
       <c r="BA107" s="173"/>
       <c r="BB107" s="291">
         <f>(AM107*0.6%)+(1*CK107)</f>
-        <v>3.3400000000000006E-2</v>
+        <v>3.2410000000000001</v>
       </c>
       <c r="BC107" s="291"/>
       <c r="BD107" s="291"/>
@@ -26588,7 +26628,7 @@
       <c r="BF107" s="291"/>
       <c r="BG107" s="291">
         <f t="shared" ref="BG107" si="171">L107+BB107</f>
-        <v>5.4334000000000007</v>
+        <v>8.641</v>
       </c>
       <c r="BH107" s="291"/>
       <c r="BI107" s="291"/>
@@ -26596,7 +26636,7 @@
       <c r="BK107" s="291"/>
       <c r="BL107" s="291">
         <f t="shared" ref="BL107" si="172">L107-BB107</f>
-        <v>5.3666</v>
+        <v>2.1590000000000003</v>
       </c>
       <c r="BM107" s="291"/>
       <c r="BN107" s="291"/>
@@ -26604,7 +26644,7 @@
       <c r="BP107" s="291"/>
       <c r="BQ107" s="292" t="str">
         <f t="shared" ref="BQ107" si="173">IF(AND(AM107&lt;=BG107,AM107&gt;=BL107),"PASS","FAIL")</f>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
       <c r="BR107" s="292"/>
       <c r="BS107" s="292"/>
@@ -26672,7 +26712,7 @@
       </c>
       <c r="CQ107" s="6">
         <f t="shared" ref="CQ107" si="180">STDEV(X107:AL107)</f>
-        <v>1.0877919644084146E-15</v>
+        <v>0</v>
       </c>
       <c r="CR107" s="1" t="str">
         <f t="shared" ref="CR107" si="181">P107</f>
@@ -26684,7 +26724,7 @@
       </c>
       <c r="CT107" s="86">
         <f t="shared" ref="CT107" si="182">CQ107/CS107</f>
-        <v>6.2803698347350997E-16</v>
+        <v>0</v>
       </c>
       <c r="CU107" s="8"/>
       <c r="CV107" s="94">
@@ -34688,628 +34728,636 @@
     <mergeCell ref="S126:W126"/>
   </mergeCells>
   <conditionalFormatting sqref="B140:T140 AK140:AZ140 B143:T143 AK143:AZ143 B146:T146 AK146:AZ147">
-    <cfRule type="notContainsBlanks" dxfId="141" priority="451">
+    <cfRule type="notContainsBlanks" dxfId="143" priority="453">
       <formula>LEN(TRIM(B140))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33:AZ34">
-    <cfRule type="notContainsBlanks" dxfId="140" priority="287">
+    <cfRule type="notContainsBlanks" dxfId="142" priority="289">
       <formula>LEN(TRIM(B33))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L55:L60">
-    <cfRule type="expression" dxfId="139" priority="232">
+    <cfRule type="expression" dxfId="141" priority="234">
       <formula>$BQ$55="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:N7 AN7:AP7 K9:AA22 AL9:AZ22 AG29:AX29 B37:AZ38 K41:L42 T41:U42 C45:AS48">
-    <cfRule type="notContainsBlanks" dxfId="138" priority="452">
+    <cfRule type="notContainsBlanks" dxfId="140" priority="454">
       <formula>LEN(TRIM(B7))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L62:O65">
-    <cfRule type="expression" dxfId="137" priority="228">
+    <cfRule type="expression" dxfId="139" priority="230">
       <formula>$BQ$61="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L70:O71">
-    <cfRule type="expression" dxfId="136" priority="146">
+    <cfRule type="expression" dxfId="138" priority="148">
       <formula>$BQ$66="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L77:O83">
-    <cfRule type="expression" dxfId="135" priority="186">
+    <cfRule type="expression" dxfId="137" priority="188">
       <formula>$BQ$80="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L85:O89">
-    <cfRule type="expression" dxfId="134" priority="181">
+    <cfRule type="expression" dxfId="136" priority="183">
       <formula>$BQ$84="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L95:O97">
-    <cfRule type="expression" dxfId="133" priority="134">
+    <cfRule type="expression" dxfId="135" priority="136">
       <formula>$BQ$90="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L113:O117">
-    <cfRule type="expression" dxfId="132" priority="36">
+    <cfRule type="expression" dxfId="134" priority="38">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L127:O133">
-    <cfRule type="expression" dxfId="131" priority="24">
+    <cfRule type="expression" dxfId="133" priority="26">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L61:R61 X61:AV61">
-    <cfRule type="expression" dxfId="130" priority="437">
+    <cfRule type="expression" dxfId="132" priority="439">
       <formula>$BQ$61="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L66:R66">
-    <cfRule type="expression" dxfId="129" priority="429">
+    <cfRule type="expression" dxfId="131" priority="431">
       <formula>$BQ$66="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L67:R67">
-    <cfRule type="expression" dxfId="128" priority="428">
+    <cfRule type="expression" dxfId="130" priority="430">
       <formula>$BQ$67="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L68:R68">
-    <cfRule type="expression" dxfId="127" priority="427">
+    <cfRule type="expression" dxfId="129" priority="429">
       <formula>$BQ$68="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L69:R69">
-    <cfRule type="expression" dxfId="126" priority="150">
+    <cfRule type="expression" dxfId="128" priority="152">
       <formula>$BQ$66="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L91:R91 X91:AV91">
-    <cfRule type="expression" dxfId="125" priority="411">
+    <cfRule type="expression" dxfId="127" priority="413">
       <formula>$BQ$91="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L93:R93 X93:AV93">
-    <cfRule type="expression" dxfId="124" priority="409">
+    <cfRule type="expression" dxfId="126" priority="411">
       <formula>$BQ$93="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L102:R102 X102:AV102">
-    <cfRule type="expression" dxfId="123" priority="408">
+    <cfRule type="expression" dxfId="125" priority="410">
       <formula>$BQ$102="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L103:R103 X103:AV103">
-    <cfRule type="expression" dxfId="122" priority="407">
+    <cfRule type="expression" dxfId="124" priority="409">
       <formula>$BQ$103="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L104:R104 X104:AV104">
-    <cfRule type="expression" dxfId="121" priority="406">
+    <cfRule type="expression" dxfId="123" priority="408">
       <formula>$BQ$104="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L105:R105 X105:AV105">
-    <cfRule type="expression" dxfId="120" priority="405">
+    <cfRule type="expression" dxfId="122" priority="407">
       <formula>$BQ$105="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L106:R107">
-    <cfRule type="expression" dxfId="119" priority="157">
+    <cfRule type="expression" dxfId="121" priority="159">
       <formula>$BQ$106="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L108:R108">
-    <cfRule type="expression" dxfId="118" priority="402">
+    <cfRule type="expression" dxfId="120" priority="404">
       <formula>$BQ$108="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L118:R121">
-    <cfRule type="expression" dxfId="117" priority="174">
+    <cfRule type="expression" dxfId="119" priority="176">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L135:R137">
-    <cfRule type="expression" dxfId="116" priority="171">
+    <cfRule type="expression" dxfId="118" priority="173">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P77:R79 L76:AV76">
-    <cfRule type="expression" dxfId="115" priority="226">
+    <cfRule type="expression" dxfId="117" priority="228">
       <formula>$BQ$80="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L84:AV84">
-    <cfRule type="expression" dxfId="114" priority="422">
+    <cfRule type="expression" dxfId="116" priority="424">
       <formula>$BQ$84="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L90:AV90">
-    <cfRule type="expression" dxfId="113" priority="412">
+    <cfRule type="expression" dxfId="115" priority="414">
       <formula>$BQ$90="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L92:AV92">
-    <cfRule type="expression" dxfId="112" priority="410">
+    <cfRule type="expression" dxfId="114" priority="412">
       <formula>$BQ$92="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L94:AV94">
-    <cfRule type="expression" dxfId="111" priority="142">
+    <cfRule type="expression" dxfId="113" priority="144">
       <formula>$BQ$90="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P127:R129 L126:AV126">
-    <cfRule type="expression" dxfId="110" priority="70">
+    <cfRule type="expression" dxfId="112" priority="72">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L134:AV134">
-    <cfRule type="expression" dxfId="109" priority="398">
+    <cfRule type="expression" dxfId="111" priority="400">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P55 X55:AV55">
-    <cfRule type="expression" dxfId="108" priority="443">
+    <cfRule type="expression" dxfId="110" priority="445">
       <formula>$BQ$55="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P56:R56 X56:AV56">
-    <cfRule type="expression" dxfId="107" priority="442">
+    <cfRule type="expression" dxfId="109" priority="444">
       <formula>$BQ$56="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P57:R57 X57:AV57">
-    <cfRule type="expression" dxfId="106" priority="441">
+    <cfRule type="expression" dxfId="108" priority="443">
       <formula>$BQ$57="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P58:R58 X58:AV58">
-    <cfRule type="expression" dxfId="105" priority="440">
+    <cfRule type="expression" dxfId="107" priority="442">
       <formula>$BQ$58="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P59:R59 X59:AV59">
-    <cfRule type="expression" dxfId="104" priority="439">
+    <cfRule type="expression" dxfId="106" priority="441">
       <formula>$BQ$59="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P60:R60 X60:AV60">
-    <cfRule type="expression" dxfId="103" priority="438">
+    <cfRule type="expression" dxfId="105" priority="440">
       <formula>$BQ$60="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P62:R62 X62:AV62">
-    <cfRule type="expression" dxfId="102" priority="436">
+    <cfRule type="expression" dxfId="104" priority="438">
       <formula>$BQ$62="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P63:R63 X63:AV63">
-    <cfRule type="expression" dxfId="101" priority="435">
+    <cfRule type="expression" dxfId="103" priority="437">
       <formula>$BQ$63="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P64:R64 X64:AV64">
-    <cfRule type="expression" dxfId="100" priority="434">
+    <cfRule type="expression" dxfId="102" priority="436">
       <formula>$BQ$64="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P65:R65 X65:AV65">
-    <cfRule type="expression" dxfId="99" priority="433">
+    <cfRule type="expression" dxfId="101" priority="435">
       <formula>$BQ$65="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P70:R70">
-    <cfRule type="expression" dxfId="98" priority="149">
+    <cfRule type="expression" dxfId="100" priority="151">
       <formula>$BQ$67="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P71:R71">
-    <cfRule type="expression" dxfId="97" priority="148">
+    <cfRule type="expression" dxfId="99" priority="150">
       <formula>$BQ$68="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P85:R85 X85:AV85">
-    <cfRule type="expression" dxfId="96" priority="421">
+    <cfRule type="expression" dxfId="98" priority="423">
       <formula>$BQ$85="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P87:R87 X87:AV87">
-    <cfRule type="expression" dxfId="95" priority="419">
+    <cfRule type="expression" dxfId="97" priority="421">
       <formula>$BQ$87="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P89:R89 X89:AV89">
-    <cfRule type="expression" dxfId="94" priority="417">
+    <cfRule type="expression" dxfId="96" priority="419">
       <formula>$BQ$89="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P95:R95 X95:AV95">
-    <cfRule type="expression" dxfId="93" priority="141">
+    <cfRule type="expression" dxfId="95" priority="143">
       <formula>$BQ$91="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P97:R97 X97:AV97">
-    <cfRule type="expression" dxfId="92" priority="139">
+    <cfRule type="expression" dxfId="94" priority="141">
       <formula>$BQ$93="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P113:R114">
-    <cfRule type="expression" dxfId="91" priority="109">
+    <cfRule type="expression" dxfId="93" priority="111">
       <formula>$BQ$121="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P115:R115">
-    <cfRule type="expression" dxfId="90" priority="132">
+    <cfRule type="expression" dxfId="92" priority="134">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P116:R116">
-    <cfRule type="expression" dxfId="89" priority="131">
+    <cfRule type="expression" dxfId="91" priority="133">
       <formula>$BQ$119="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P117:R117">
-    <cfRule type="expression" dxfId="88" priority="125">
+    <cfRule type="expression" dxfId="90" priority="127">
       <formula>$BQ$121="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P132:R132">
-    <cfRule type="expression" dxfId="87" priority="101">
+    <cfRule type="expression" dxfId="89" priority="103">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P133:R133">
-    <cfRule type="expression" dxfId="86" priority="100">
+    <cfRule type="expression" dxfId="88" priority="102">
       <formula>$BQ$137="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P80:AV80">
-    <cfRule type="expression" dxfId="85" priority="426">
+    <cfRule type="expression" dxfId="87" priority="428">
       <formula>$BQ$80="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P81:AV81">
-    <cfRule type="expression" dxfId="84" priority="167">
+    <cfRule type="expression" dxfId="86" priority="169">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P82:AV82">
-    <cfRule type="expression" dxfId="83" priority="424">
+    <cfRule type="expression" dxfId="85" priority="426">
       <formula>$BQ$82="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P86:AV86">
-    <cfRule type="expression" dxfId="82" priority="420">
+    <cfRule type="expression" dxfId="84" priority="422">
       <formula>$BQ$86="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P88:AV88">
-    <cfRule type="expression" dxfId="81" priority="418">
+    <cfRule type="expression" dxfId="83" priority="420">
       <formula>$BQ$88="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P96:AV96">
-    <cfRule type="expression" dxfId="80" priority="140">
+    <cfRule type="expression" dxfId="82" priority="142">
       <formula>$BQ$92="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P130:AV130">
-    <cfRule type="expression" dxfId="79" priority="103">
+    <cfRule type="expression" dxfId="81" priority="105">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P131:AV131">
-    <cfRule type="expression" dxfId="78" priority="29">
+    <cfRule type="expression" dxfId="80" priority="31">
       <formula>$BQ$135="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S79:W79">
-    <cfRule type="expression" dxfId="77" priority="168">
+    <cfRule type="expression" dxfId="79" priority="170">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S83:W83">
+    <cfRule type="expression" dxfId="78" priority="168">
+      <formula>$BQ$81="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S85:W85">
+    <cfRule type="expression" dxfId="77" priority="167">
+      <formula>$BQ$81="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S87:W87">
     <cfRule type="expression" dxfId="76" priority="166">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S85:W85">
+  <conditionalFormatting sqref="S89:W89">
     <cfRule type="expression" dxfId="75" priority="165">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S87:W87">
+  <conditionalFormatting sqref="S91:W91">
     <cfRule type="expression" dxfId="74" priority="164">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S89:W89">
+  <conditionalFormatting sqref="S93:W93">
     <cfRule type="expression" dxfId="73" priority="163">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S91:W91">
-    <cfRule type="expression" dxfId="72" priority="162">
-      <formula>$BQ$81="FAIL"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S93:W93">
-    <cfRule type="expression" dxfId="71" priority="161">
-      <formula>$BQ$81="FAIL"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="S95:W95">
-    <cfRule type="expression" dxfId="70" priority="138">
+    <cfRule type="expression" dxfId="72" priority="140">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S97:W97">
-    <cfRule type="expression" dxfId="69" priority="137">
+    <cfRule type="expression" dxfId="71" priority="139">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S128:W128">
-    <cfRule type="expression" dxfId="68" priority="42">
+    <cfRule type="expression" dxfId="70" priority="44">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S129:W129">
-    <cfRule type="expression" dxfId="67" priority="32">
+    <cfRule type="expression" dxfId="69" priority="34">
       <formula>$BQ$135="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S132:W132">
-    <cfRule type="expression" dxfId="66" priority="75">
+    <cfRule type="expression" dxfId="68" priority="77">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S133:W133">
+    <cfRule type="expression" dxfId="67" priority="30">
+      <formula>$BQ$135="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S136:W136">
+    <cfRule type="expression" dxfId="66" priority="172">
+      <formula>$BQ$134="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S137:W137">
     <cfRule type="expression" dxfId="65" priority="28">
       <formula>$BQ$135="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S136:W136">
-    <cfRule type="expression" dxfId="64" priority="170">
-      <formula>$BQ$134="FAIL"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S137:W137">
-    <cfRule type="expression" dxfId="63" priority="26">
-      <formula>$BQ$135="FAIL"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="S77:AV77">
-    <cfRule type="expression" dxfId="62" priority="225">
+    <cfRule type="expression" dxfId="64" priority="227">
       <formula>$BQ$81="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S78:AV78">
-    <cfRule type="expression" dxfId="61" priority="224">
+    <cfRule type="expression" dxfId="63" priority="226">
       <formula>$BQ$82="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S127:AV127">
-    <cfRule type="expression" dxfId="60" priority="69">
+    <cfRule type="expression" dxfId="62" priority="71">
       <formula>$BQ$135="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S135:AV135">
-    <cfRule type="expression" dxfId="59" priority="27">
+    <cfRule type="expression" dxfId="61" priority="29">
       <formula>$BQ$135="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X55:AL71">
-    <cfRule type="notContainsBlanks" dxfId="58" priority="156">
+    <cfRule type="notContainsBlanks" dxfId="60" priority="158">
       <formula>LEN(TRIM(X55))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X76:AL97">
-    <cfRule type="notContainsBlanks" dxfId="57" priority="145">
+    <cfRule type="notContainsBlanks" dxfId="59" priority="147">
       <formula>LEN(TRIM(X76))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X79:AL79">
-    <cfRule type="expression" dxfId="56" priority="15">
+    <cfRule type="expression" dxfId="58" priority="17">
       <formula>$BQ$82="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X83:AL83">
-    <cfRule type="expression" dxfId="55" priority="13">
+    <cfRule type="expression" dxfId="57" priority="15">
       <formula>$BQ$82="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X102:AL108">
-    <cfRule type="notContainsBlanks" dxfId="54" priority="160">
+    <cfRule type="notContainsBlanks" dxfId="56" priority="162">
       <formula>LEN(TRIM(X102))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X113:AL121">
-    <cfRule type="notContainsBlanks" dxfId="53" priority="11">
+    <cfRule type="notContainsBlanks" dxfId="55" priority="13">
       <formula>LEN(TRIM(X113))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X119:AL121">
-    <cfRule type="expression" dxfId="52" priority="9">
+    <cfRule type="expression" dxfId="54" priority="11">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X120:AL121">
-    <cfRule type="expression" dxfId="51" priority="10">
+    <cfRule type="expression" dxfId="53" priority="12">
       <formula>$BQ$119="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X126:AL137">
-    <cfRule type="notContainsBlanks" dxfId="50" priority="71">
+    <cfRule type="notContainsBlanks" dxfId="52" priority="73">
       <formula>LEN(TRIM(X126))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X129:AL129">
-    <cfRule type="expression" dxfId="49" priority="4">
+    <cfRule type="expression" dxfId="51" priority="6">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X133:AL133">
-    <cfRule type="expression" dxfId="48" priority="6">
+    <cfRule type="expression" dxfId="50" priority="8">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X135:AL137">
-    <cfRule type="expression" dxfId="47" priority="5">
+    <cfRule type="expression" dxfId="49" priority="7">
       <formula>$BQ$134="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X137:AL137">
-    <cfRule type="expression" dxfId="46" priority="19">
+    <cfRule type="expression" dxfId="48" priority="21">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X66:AV66">
-    <cfRule type="expression" dxfId="45" priority="432">
+    <cfRule type="expression" dxfId="47" priority="434">
       <formula>$BQ$66="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X67:AV67">
-    <cfRule type="expression" dxfId="44" priority="431">
+    <cfRule type="expression" dxfId="46" priority="433">
       <formula>$BQ$67="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X68:AV68">
-    <cfRule type="expression" dxfId="43" priority="430">
+    <cfRule type="expression" dxfId="45" priority="432">
       <formula>$BQ$68="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X69:AV69">
-    <cfRule type="expression" dxfId="42" priority="153">
+    <cfRule type="expression" dxfId="44" priority="155">
       <formula>$BQ$66="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X70:AV70">
-    <cfRule type="expression" dxfId="41" priority="152">
+    <cfRule type="expression" dxfId="43" priority="154">
       <formula>$BQ$67="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X71:AV71">
-    <cfRule type="expression" dxfId="40" priority="151">
+    <cfRule type="expression" dxfId="42" priority="153">
       <formula>$BQ$68="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P83:R83 X79:AV79 X83:AV83">
-    <cfRule type="expression" dxfId="39" priority="423">
+    <cfRule type="expression" dxfId="41" priority="425">
       <formula>$BQ$83="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X106:AV107">
-    <cfRule type="expression" dxfId="38" priority="404">
+    <cfRule type="expression" dxfId="40" priority="406">
       <formula>$BQ$106="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X108:AV108">
-    <cfRule type="expression" dxfId="37" priority="403">
+    <cfRule type="expression" dxfId="39" priority="405">
       <formula>$BQ$108="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X113:AV113">
-    <cfRule type="expression" dxfId="36" priority="120">
+    <cfRule type="expression" dxfId="38" priority="122">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X114:AV114">
-    <cfRule type="expression" dxfId="35" priority="118">
+    <cfRule type="expression" dxfId="37" priority="120">
       <formula>$BQ$121="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X115:AV115 X118:AV118">
-    <cfRule type="expression" dxfId="34" priority="401">
+    <cfRule type="expression" dxfId="36" priority="403">
       <formula>$BQ$118="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X116:AV116 X119:AV119">
-    <cfRule type="expression" dxfId="33" priority="400">
+    <cfRule type="expression" dxfId="35" priority="402">
       <formula>$BQ$119="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM120:AV121 X117:AV117">
-    <cfRule type="expression" dxfId="32" priority="399">
+    <cfRule type="expression" dxfId="34" priority="401">
       <formula>$BQ$121="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X128:AV128">
-    <cfRule type="expression" dxfId="31" priority="73">
+    <cfRule type="expression" dxfId="33" priority="75">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X129:AV129">
-    <cfRule type="expression" dxfId="30" priority="72">
+    <cfRule type="expression" dxfId="32" priority="74">
       <formula>$BQ$137="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X132:AV132 X136:AV136">
-    <cfRule type="expression" dxfId="29" priority="396">
+    <cfRule type="expression" dxfId="31" priority="398">
       <formula>$BQ$136="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X133:AV133 X137:AV137">
-    <cfRule type="expression" dxfId="28" priority="395">
+    <cfRule type="expression" dxfId="30" priority="397">
       <formula>$BQ$137="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="BQ55:BU71">
-    <cfRule type="containsText" dxfId="27" priority="154" operator="containsText" text="PASS">
-      <formula>NOT(ISERROR(SEARCH("PASS",BQ55)))</formula>
+  <conditionalFormatting sqref="BQ56:BU71">
+    <cfRule type="containsText" dxfId="29" priority="156" operator="containsText" text="PASS">
+      <formula>NOT(ISERROR(SEARCH("PASS",BQ56)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="155" operator="containsText" text="FAIL">
-      <formula>NOT(ISERROR(SEARCH("FAIL",BQ55)))</formula>
+    <cfRule type="containsText" dxfId="28" priority="157" operator="containsText" text="FAIL">
+      <formula>NOT(ISERROR(SEARCH("FAIL",BQ56)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BQ76:BU97">
-    <cfRule type="containsText" dxfId="25" priority="144" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="27" priority="146" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",BQ76)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="143" operator="containsText" text="PASS">
+    <cfRule type="containsText" dxfId="26" priority="145" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",BQ76)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BQ102:BU108">
-    <cfRule type="containsText" dxfId="23" priority="158" operator="containsText" text="PASS">
+    <cfRule type="containsText" dxfId="25" priority="160" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",BQ102)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="159" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="24" priority="161" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",BQ102)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BQ113:BU121">
-    <cfRule type="containsText" dxfId="21" priority="108" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="23" priority="110" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",BQ113)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="107" operator="containsText" text="PASS">
+    <cfRule type="containsText" dxfId="22" priority="109" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",BQ113)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BQ126:BU137">
-    <cfRule type="containsText" dxfId="19" priority="66" operator="containsText" text="FAIL">
+    <cfRule type="containsText" dxfId="21" priority="68" operator="containsText" text="FAIL">
       <formula>NOT(ISERROR(SEARCH("FAIL",BQ126)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="65" operator="containsText" text="PASS">
+    <cfRule type="containsText" dxfId="20" priority="67" operator="containsText" text="PASS">
       <formula>NOT(ISERROR(SEARCH("PASS",BQ126)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X57:AL57">
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="19" priority="5">
       <formula>$BQ$56="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="X77:AB77">
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="18" priority="4">
       <formula>$BQ$80="FAIL"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC77:AL77">
-    <cfRule type="expression" dxfId="15" priority="1">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>$BQ$80="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="BQ55:BU55">
+    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="PASS">
+      <formula>NOT(ISERROR(SEARCH("PASS",BQ55)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="FAIL">
+      <formula>NOT(ISERROR(SEARCH("FAIL",BQ55)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -35577,95 +35625,95 @@
       <c r="Y9" s="460"/>
     </row>
     <row r="10" spans="2:25">
-      <c r="B10" s="43" t="e">
+      <c r="B10" s="43">
         <f>DataSheet!AM55</f>
-        <v>#DIV/0!</v>
+        <v>60</v>
       </c>
       <c r="C10" s="44" t="str">
         <f>DataSheet!P55</f>
         <v>mV</v>
       </c>
-      <c r="D10" s="51" t="e">
+      <c r="D10" s="51">
         <f>ABS((B10*0.7%)+(3*DataSheet!CK55))</f>
-        <v>#DIV/0!</v>
+        <v>0.72</v>
       </c>
       <c r="E10" s="35" t="str">
         <f>C10</f>
         <v>mV</v>
       </c>
-      <c r="F10" s="38" t="e">
+      <c r="F10" s="38">
         <f>DataSheet!DD55</f>
-        <v>#DIV/0!</v>
+        <v>5.7740161355276223E-2</v>
       </c>
       <c r="G10" s="35" t="str">
         <f>E10</f>
         <v>mV</v>
       </c>
-      <c r="H10" s="39" t="e">
+      <c r="H10" s="39">
         <f>DataSheet!L55+D10</f>
-        <v>#DIV/0!</v>
+        <v>60.72</v>
       </c>
       <c r="I10" s="35" t="str">
         <f>G10</f>
         <v>mV</v>
       </c>
-      <c r="J10" s="39" t="e">
+      <c r="J10" s="39">
         <f>DataSheet!L55-D10</f>
-        <v>#DIV/0!</v>
+        <v>59.28</v>
       </c>
       <c r="K10" s="35" t="str">
         <f>I10</f>
         <v>mV</v>
       </c>
-      <c r="L10" s="480" t="e">
+      <c r="L10" s="480" t="str">
         <f>IF(AND(B10&lt;=H10,B10&gt;=J10),"PASSED","FAILED")</f>
-        <v>#DIV/0!</v>
+        <v>PASSED</v>
       </c>
       <c r="M10" s="480"/>
-      <c r="N10" s="39" t="e">
+      <c r="N10" s="39">
         <f>F10+B10</f>
-        <v>#DIV/0!</v>
+        <v>60.057740161355277</v>
       </c>
       <c r="O10" s="40" t="str">
         <f>G10</f>
         <v>mV</v>
       </c>
-      <c r="P10" s="39" t="e">
+      <c r="P10" s="39">
         <f>H10</f>
-        <v>#DIV/0!</v>
+        <v>60.72</v>
       </c>
       <c r="Q10" s="35" t="str">
         <f>O10</f>
         <v>mV</v>
       </c>
-      <c r="R10" s="474" t="e">
+      <c r="R10" s="474" t="str">
         <f>IF(AND(N10&lt;=H10,N10&gt;=J10),"PASSED","FAILED")</f>
-        <v>#DIV/0!</v>
+        <v>PASSED</v>
       </c>
       <c r="S10" s="474"/>
-      <c r="T10" s="39" t="e">
+      <c r="T10" s="39">
         <f>-F10+B10</f>
-        <v>#DIV/0!</v>
+        <v>59.942259838644723</v>
       </c>
       <c r="U10" s="37" t="str">
         <f>O10</f>
         <v>mV</v>
       </c>
-      <c r="V10" s="472" t="e">
+      <c r="V10" s="472" t="str">
         <f>IF(AND(T10&lt;=H10,T10&gt;=J10),"PASSED","FAILED")</f>
-        <v>#DIV/0!</v>
+        <v>PASSED</v>
       </c>
       <c r="W10" s="472"/>
-      <c r="X10" s="471" t="e">
+      <c r="X10" s="471" t="str">
         <f t="shared" ref="X10:X26" si="0">IF(AND(L10="PASSED",R10="PASSED",V10="PASSED"),"PASSED",IF(L10="FAILED","FAILED","UNDETERMINED"))</f>
-        <v>#DIV/0!</v>
+        <v>PASSED</v>
       </c>
       <c r="Y10" s="471"/>
     </row>
     <row r="11" spans="2:25">
       <c r="B11" s="43">
         <f>DataSheet!AM56</f>
-        <v>40</v>
+        <v>540</v>
       </c>
       <c r="C11" s="44" t="str">
         <f>DataSheet!P56</f>
@@ -35673,7 +35721,7 @@
       </c>
       <c r="D11" s="51">
         <f>ABS((B11*0.7%)+(3*DataSheet!CK56))</f>
-        <v>0.58000000000000007</v>
+        <v>4.08</v>
       </c>
       <c r="E11" s="35" t="str">
         <f t="shared" ref="E11:E26" si="1">C11</f>
@@ -35681,7 +35729,7 @@
       </c>
       <c r="F11" s="38">
         <f>DataSheet!DD56</f>
-        <v>80.000083443539822</v>
+        <v>5.7773206015707089E-2</v>
       </c>
       <c r="G11" s="35" t="str">
         <f t="shared" ref="G11:G26" si="2">E11</f>
@@ -35689,7 +35737,7 @@
       </c>
       <c r="H11" s="39">
         <f>DataSheet!L56+D11</f>
-        <v>540.58000000000004</v>
+        <v>544.08000000000004</v>
       </c>
       <c r="I11" s="35" t="str">
         <f t="shared" ref="I11:I26" si="3">G11</f>
@@ -35697,7 +35745,7 @@
       </c>
       <c r="J11" s="39">
         <f>DataSheet!L56-D11</f>
-        <v>539.41999999999996</v>
+        <v>535.91999999999996</v>
       </c>
       <c r="K11" s="35" t="str">
         <f t="shared" ref="K11:K26" si="4">I11</f>
@@ -35705,12 +35753,12 @@
       </c>
       <c r="L11" s="480" t="str">
         <f t="shared" ref="L11:L26" si="5">IF(AND(B11&lt;=H11,B11&gt;=J11),"PASSED","FAILED")</f>
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="M11" s="480"/>
       <c r="N11" s="39">
         <f t="shared" ref="N11:N12" si="6">F11+B11</f>
-        <v>120.00008344353982</v>
+        <v>540.05777320601567</v>
       </c>
       <c r="O11" s="40" t="str">
         <f t="shared" ref="O11:O26" si="7">G11</f>
@@ -35718,7 +35766,7 @@
       </c>
       <c r="P11" s="39">
         <f t="shared" ref="P11:P12" si="8">H11</f>
-        <v>540.58000000000004</v>
+        <v>544.08000000000004</v>
       </c>
       <c r="Q11" s="35" t="str">
         <f t="shared" ref="Q11:Q26" si="9">O11</f>
@@ -35726,12 +35774,12 @@
       </c>
       <c r="R11" s="474" t="str">
         <f t="shared" ref="R11:R26" si="10">IF(AND(N11&lt;=H11,N11&gt;=J11),"PASSED","FAILED")</f>
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="S11" s="474"/>
       <c r="T11" s="39">
         <f t="shared" ref="T11:T12" si="11">-F11+B11</f>
-        <v>-40.000083443539822</v>
+        <v>539.94222679398433</v>
       </c>
       <c r="U11" s="37" t="str">
         <f t="shared" ref="U11:U26" si="12">O11</f>
@@ -35739,12 +35787,12 @@
       </c>
       <c r="V11" s="472" t="str">
         <f t="shared" ref="V11:V26" si="13">IF(AND(T11&lt;=H11,T11&gt;=J11),"PASSED","FAILED")</f>
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="W11" s="472"/>
       <c r="X11" s="471" t="str">
         <f t="shared" si="0"/>
-        <v>FAILED</v>
+        <v>PASSED</v>
       </c>
       <c r="Y11" s="471"/>
     </row>

</xml_diff>